<commit_message>
feat: add component reuse, automotive and battery BMS skills
</commit_message>
<xml_diff>
--- a/agent-unified/docs/技能与MCP维护清单-公开版.xlsx
+++ b/agent-unified/docs/技能与MCP维护清单-公开版.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="技能清单" sheetId="1" r:id="Ra52ec2f50c0b42e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP清单" sheetId="2" r:id="R82109f8dbc7347f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="平台工具" sheetId="3" r:id="R4c86e5f25f4c4e30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="4" r:id="R8941bc6f05db468c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="技能清单" sheetId="1" r:id="R9b6e1c83611648ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP清单" sheetId="2" r:id="Rdc7efc4afb5b4d4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="平台工具" sheetId="3" r:id="R9f2dead455ae4f4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新记录" sheetId="4" r:id="R77300e139c934d1e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="201" formatCode="&quot;核对日期：&quot;yyyy-mm-dd"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -87,7 +88,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -130,6 +131,9 @@
     <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -160,8 +164,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SkillInventory" displayName="SkillInventory" ref="A7:O74" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:O74"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SkillInventory" displayName="SkillInventory" ref="A7:O77" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:O77"/>
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="名称"/>
@@ -475,7 +479,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>2026-10-15 维护快照。记录包含客户端与第三方能力，登记不代表公开包已安装。</x:v>
+        <x:v>2026-10-16 增补组件复用、车载嵌入式与 BMS 技能；其余条目保留各自最近核对日期。</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -518,10 +522,10 @@
       <x:c r="B4" s="3"/>
       <x:c r="C4" s="6" t="n">
         <x:f>COUNTA(A8:A1000)</x:f>
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="D4" s="3" t="str">
-        <x:v>核对日期：2026-10-15</x:v>
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E4" s="3"/>
       <x:c r="F4" s="3" t="str">
@@ -3510,6 +3514,141 @@
       </x:c>
       <x:c r="O74" s="9" t="str">
         <x:v>公开版内置，随仓库提供。未安装额外 SDK/驱动；未编译实际工程或操作目标设备</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="112" customHeight="1">
+      <x:c r="A75" s="9" t="str">
+        <x:v>SK-068</x:v>
+      </x:c>
+      <x:c r="B75" s="9" t="str">
+        <x:v>component-reuse</x:v>
+      </x:c>
+      <x:c r="C75" s="9" t="str">
+        <x:v>个人技能</x:v>
+      </x:c>
+      <x:c r="D75" s="9" t="str">
+        <x:v>旧代码提取、上游选型、平台解耦与接入验证</x:v>
+      </x:c>
+      <x:c r="E75" s="9" t="str">
+        <x:v>技能 1.0.0；SHA256 64e345f65221</x:v>
+      </x:c>
+      <x:c r="F75" s="9" t="str">
+        <x:v>已登记；目标环境需验证</x:v>
+      </x:c>
+      <x:c r="G75" s="9" t="str">
+        <x:v>Windows/Linux 规则共用</x:v>
+      </x:c>
+      <x:c r="H75" s="9" t="str">
+        <x:v>随迁移包或源码安装器更新</x:v>
+      </x:c>
+      <x:c r="I75" s="11" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J75" s="12" t="str"/>
+      <x:c r="K75" s="12" t="str">
+        <x:v>已更新</x:v>
+      </x:c>
+      <x:c r="L75" s="12" t="str">
+        <x:v>含 GitHub 候选目录；未批量安装候选代码</x:v>
+      </x:c>
+      <x:c r="M75" s="9" t="str">
+        <x:v>agent-unified/payload/skills/component-reuse</x:v>
+      </x:c>
+      <x:c r="N75" s="9" t="str">
+        <x:v>GitHub 快照见 references/github-snapshot.json</x:v>
+      </x:c>
+      <x:c r="O75" s="9" t="str">
+        <x:v>公开版内置。真实目标/硬件需验证；标准引用不转授版权</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="112" customHeight="1">
+      <x:c r="A76" s="9" t="str">
+        <x:v>SK-069</x:v>
+      </x:c>
+      <x:c r="B76" s="9" t="str">
+        <x:v>automotive-embedded-engineering</x:v>
+      </x:c>
+      <x:c r="C76" s="9" t="str">
+        <x:v>个人技能</x:v>
+      </x:c>
+      <x:c r="D76" s="9" t="str">
+        <x:v>ECU、AUTOSAR、车载通信诊断、安全升级与工程证据</x:v>
+      </x:c>
+      <x:c r="E76" s="9" t="str">
+        <x:v>技能 1.0.0；SHA256 0bb2e66eb765</x:v>
+      </x:c>
+      <x:c r="F76" s="9" t="str">
+        <x:v>已登记；目标环境需验证</x:v>
+      </x:c>
+      <x:c r="G76" s="9" t="str">
+        <x:v>Windows/Linux 规则共用</x:v>
+      </x:c>
+      <x:c r="H76" s="9" t="str">
+        <x:v>随迁移包或源码安装器更新</x:v>
+      </x:c>
+      <x:c r="I76" s="11" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J76" s="12" t="str"/>
+      <x:c r="K76" s="12" t="str">
+        <x:v>已更新</x:v>
+      </x:c>
+      <x:c r="L76" s="12" t="str">
+        <x:v>原创规则；官方来源按任务读取</x:v>
+      </x:c>
+      <x:c r="M76" s="9" t="str">
+        <x:v>agent-unified/payload/skills/automotive-embedded-engineering</x:v>
+      </x:c>
+      <x:c r="N76" s="9" t="str">
+        <x:v>官方题录与核实范围见 references/standards.md</x:v>
+      </x:c>
+      <x:c r="O76" s="9" t="str">
+        <x:v>公开版内置。真实目标/硬件需验证；标准引用不转授版权</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="112" customHeight="1">
+      <x:c r="A77" s="9" t="str">
+        <x:v>SK-070</x:v>
+      </x:c>
+      <x:c r="B77" s="9" t="str">
+        <x:v>battery-bms-engineering</x:v>
+      </x:c>
+      <x:c r="C77" s="9" t="str">
+        <x:v>个人技能</x:v>
+      </x:c>
+      <x:c r="D77" s="9" t="str">
+        <x:v>动力及储能 BMS、采样估算、均衡热管理与保护验证</x:v>
+      </x:c>
+      <x:c r="E77" s="9" t="str">
+        <x:v>技能 1.0.0；SHA256 500cf7f7f49d</x:v>
+      </x:c>
+      <x:c r="F77" s="9" t="str">
+        <x:v>已登记；目标环境需验证</x:v>
+      </x:c>
+      <x:c r="G77" s="9" t="str">
+        <x:v>Windows/Linux 规则共用</x:v>
+      </x:c>
+      <x:c r="H77" s="9" t="str">
+        <x:v>随迁移包或源码安装器更新</x:v>
+      </x:c>
+      <x:c r="I77" s="11" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J77" s="12" t="str"/>
+      <x:c r="K77" s="12" t="str">
+        <x:v>已更新</x:v>
+      </x:c>
+      <x:c r="L77" s="12" t="str">
+        <x:v>原创规则；官方来源按任务读取</x:v>
+      </x:c>
+      <x:c r="M77" s="9" t="str">
+        <x:v>agent-unified/payload/skills/battery-bms-engineering</x:v>
+      </x:c>
+      <x:c r="N77" s="9" t="str">
+        <x:v>官方题录与核实范围见 references/standards.md</x:v>
+      </x:c>
+      <x:c r="O77" s="9" t="str">
+        <x:v>公开版内置。真实目标/硬件需验证；标准引用不转授版权</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3530,7 +3669,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d19e54638c84f78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6907eafacefd40e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3913,7 +4052,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd69739fa7c5346b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2234ae9225640a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4509,7 +4648,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2374d46d242e4fdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcad4382ad2d8464f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4544,7 +4683,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>2026-10-15 维护快照。记录包含客户端与第三方能力，登记不代表公开包已安装。</x:v>
+        <x:v>2026-10-16 增补组件复用、车载嵌入式与 BMS 技能；其余条目保留各自最近核对日期。</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -4575,10 +4714,10 @@
       <x:c r="B4" s="3"/>
       <x:c r="C4" s="6" t="n">
         <x:f>COUNTA(A8:A1000)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="D4" s="3" t="str">
-        <x:v>核对日期：2026-10-15</x:v>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E4" s="3"/>
       <x:c r="F4" s="3"/>
@@ -4809,38 +4948,92 @@
         <x:v>Codex</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="52" customHeight="1">
-      <x:c r="A14" s="12"/>
-      <x:c r="B14" s="14"/>
-      <x:c r="C14" s="12"/>
-      <x:c r="D14" s="12"/>
-      <x:c r="E14" s="12"/>
-      <x:c r="F14" s="12"/>
-      <x:c r="G14" s="12"/>
-      <x:c r="H14" s="12"/>
-      <x:c r="I14" s="12"/>
-    </x:row>
-    <x:row r="15" ht="52" customHeight="1">
-      <x:c r="A15" s="12"/>
-      <x:c r="B15" s="14"/>
-      <x:c r="C15" s="12"/>
-      <x:c r="D15" s="12"/>
-      <x:c r="E15" s="12"/>
-      <x:c r="F15" s="12"/>
-      <x:c r="G15" s="12"/>
-      <x:c r="H15" s="12"/>
-      <x:c r="I15" s="12"/>
-    </x:row>
-    <x:row r="16" ht="52" customHeight="1">
-      <x:c r="A16" s="12"/>
-      <x:c r="B16" s="14"/>
-      <x:c r="C16" s="12"/>
-      <x:c r="D16" s="12"/>
-      <x:c r="E16" s="12"/>
-      <x:c r="F16" s="12"/>
-      <x:c r="G16" s="12"/>
-      <x:c r="H16" s="12"/>
-      <x:c r="I16" s="12"/>
+    <x:row r="14" ht="70" customHeight="1">
+      <x:c r="A14" s="12" t="str">
+        <x:v>LOG-007</x:v>
+      </x:c>
+      <x:c r="B14" s="14" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C14" s="12" t="str">
+        <x:v>component-reuse</x:v>
+      </x:c>
+      <x:c r="D14" s="12" t="str">
+        <x:v>新增</x:v>
+      </x:c>
+      <x:c r="E14" s="12" t="str">
+        <x:v>未登记</x:v>
+      </x:c>
+      <x:c r="F14" s="12" t="str">
+        <x:v>1.0.0</x:v>
+      </x:c>
+      <x:c r="G14" s="12" t="str">
+        <x:v>结构、链接、安装回退验证</x:v>
+      </x:c>
+      <x:c r="H14" s="12" t="str">
+        <x:v>补登记组件复用技能；候选代码未批量安装</x:v>
+      </x:c>
+      <x:c r="I14" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="70" customHeight="1">
+      <x:c r="A15" s="12" t="str">
+        <x:v>LOG-008</x:v>
+      </x:c>
+      <x:c r="B15" s="14" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C15" s="12" t="str">
+        <x:v>automotive-embedded-engineering</x:v>
+      </x:c>
+      <x:c r="D15" s="12" t="str">
+        <x:v>新增</x:v>
+      </x:c>
+      <x:c r="E15" s="12" t="str">
+        <x:v>未登记</x:v>
+      </x:c>
+      <x:c r="F15" s="12" t="str">
+        <x:v>1.0.0</x:v>
+      </x:c>
+      <x:c r="G15" s="12" t="str">
+        <x:v>结构、链接、安装回退验证</x:v>
+      </x:c>
+      <x:c r="H15" s="12" t="str">
+        <x:v>新增专项规则与官方来源；真实目标未验证</x:v>
+      </x:c>
+      <x:c r="I15" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="70" customHeight="1">
+      <x:c r="A16" s="12" t="str">
+        <x:v>LOG-009</x:v>
+      </x:c>
+      <x:c r="B16" s="14" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C16" s="12" t="str">
+        <x:v>battery-bms-engineering</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="str">
+        <x:v>新增</x:v>
+      </x:c>
+      <x:c r="E16" s="12" t="str">
+        <x:v>未登记</x:v>
+      </x:c>
+      <x:c r="F16" s="12" t="str">
+        <x:v>1.0.0</x:v>
+      </x:c>
+      <x:c r="G16" s="12" t="str">
+        <x:v>结构、链接、安装回退验证</x:v>
+      </x:c>
+      <x:c r="H16" s="12" t="str">
+        <x:v>新增专项规则与官方来源；真实目标未验证</x:v>
+      </x:c>
+      <x:c r="I16" s="12" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="52" customHeight="1">
       <x:c r="A17" s="12"/>
@@ -7841,7 +8034,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcef989e5fd3a4bf9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R092a0642b8e747b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>